<commit_message>
Beam C-Channel: show beam length in feet on offer sheet
Add length_ft (length rounded up to nearest foot) and use it in the offer
instead of length_m; template header relabelled m -> ft. Other calcs keep
using the metre columns.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/reference_xls/offer_templates/beam_c_channel.xlsx
+++ b/src/reference_xls/offer_templates/beam_c_channel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/snigdhagoel/Documents/Vibrant Technik/vibrant-technik/material-calculator/reference_xls/offer_templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/snigdhagoel/Documents/Vibrant Technik/vibrant-technik/tabular-entry/src/reference_xls/offer_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E0D296D-0C36-144F-8405-0AF113E51C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EB1B23F-0510-014B-A6EC-F0C55D78DE2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15940" xr2:uid="{8427CCFC-2C3B-484F-AD5C-2D86451F50CF}"/>
   </bookViews>
@@ -44,9 +44,6 @@
     <t>Width (mm)</t>
   </si>
   <si>
-    <t>Total Product Length (m)</t>
-  </si>
-  <si>
     <t>Area Name</t>
   </si>
   <si>
@@ -57,6 +54,9 @@
   </si>
   <si>
     <t>Beam C-Channel</t>
+  </si>
+  <si>
+    <t>Total Product Length (ft)</t>
   </si>
 </sst>
 </file>
@@ -148,12 +148,6 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -162,17 +156,23 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -511,327 +511,327 @@
   <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="6" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="11.1640625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="12.5" style="4" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="10.83203125" style="4"/>
+    <col min="1" max="1" width="6" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.1640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.5" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" ht="30" customHeight="1">
+      <c r="A2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="3"/>
+    </row>
+    <row r="3" spans="1:7" ht="49" customHeight="1">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="3"/>
-    </row>
-    <row r="2" spans="1:7" ht="30" customHeight="1">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row r="3" spans="1:7" ht="49" customHeight="1">
-      <c r="A3" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="4" spans="1:7" ht="30" customHeight="1">
-      <c r="F4" s="6"/>
+      <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:7" ht="30" customHeight="1">
-      <c r="F5" s="6"/>
+      <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:7" ht="30" customHeight="1">
-      <c r="F6" s="6"/>
+      <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:7" ht="30" customHeight="1">
-      <c r="F7" s="6"/>
+      <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:7" ht="30" customHeight="1">
-      <c r="F8" s="6"/>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:7" ht="30" customHeight="1">
-      <c r="F9" s="6"/>
+      <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:7" ht="30" customHeight="1">
-      <c r="F10" s="6"/>
+      <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:7" ht="30" customHeight="1">
-      <c r="F11" s="6"/>
+      <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:7" ht="30" customHeight="1">
-      <c r="F12" s="6"/>
+      <c r="F12" s="4"/>
     </row>
     <row r="13" spans="1:7" ht="30" customHeight="1">
-      <c r="F13" s="6"/>
+      <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:7" ht="30" customHeight="1">
-      <c r="F14" s="6"/>
+      <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:7" ht="30" customHeight="1">
-      <c r="F15" s="6"/>
+      <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:7" ht="30" customHeight="1">
-      <c r="F16" s="6"/>
+      <c r="F16" s="4"/>
     </row>
     <row r="17" spans="6:6" ht="30" customHeight="1">
-      <c r="F17" s="6"/>
+      <c r="F17" s="4"/>
     </row>
     <row r="18" spans="6:6" ht="30" customHeight="1">
-      <c r="F18" s="6"/>
+      <c r="F18" s="4"/>
     </row>
     <row r="19" spans="6:6" ht="30" customHeight="1">
-      <c r="F19" s="6"/>
+      <c r="F19" s="4"/>
     </row>
     <row r="20" spans="6:6" ht="30" customHeight="1">
-      <c r="F20" s="6"/>
+      <c r="F20" s="4"/>
     </row>
     <row r="21" spans="6:6" ht="30" customHeight="1">
-      <c r="F21" s="6"/>
+      <c r="F21" s="4"/>
     </row>
     <row r="22" spans="6:6" ht="30" customHeight="1">
-      <c r="F22" s="6"/>
+      <c r="F22" s="4"/>
     </row>
     <row r="23" spans="6:6" ht="30" customHeight="1">
-      <c r="F23" s="6"/>
+      <c r="F23" s="4"/>
     </row>
     <row r="24" spans="6:6" ht="30" customHeight="1">
-      <c r="F24" s="6"/>
+      <c r="F24" s="4"/>
     </row>
     <row r="25" spans="6:6" ht="30" customHeight="1">
-      <c r="F25" s="6"/>
+      <c r="F25" s="4"/>
     </row>
     <row r="26" spans="6:6" ht="30" customHeight="1">
-      <c r="F26" s="6"/>
+      <c r="F26" s="4"/>
     </row>
     <row r="27" spans="6:6" ht="30" customHeight="1">
-      <c r="F27" s="6"/>
+      <c r="F27" s="4"/>
     </row>
     <row r="28" spans="6:6" ht="30" customHeight="1">
-      <c r="F28" s="6"/>
+      <c r="F28" s="4"/>
     </row>
     <row r="29" spans="6:6" ht="30" customHeight="1">
-      <c r="F29" s="6"/>
+      <c r="F29" s="4"/>
     </row>
     <row r="30" spans="6:6" ht="30" customHeight="1">
-      <c r="F30" s="6"/>
+      <c r="F30" s="4"/>
     </row>
     <row r="31" spans="6:6" ht="30" customHeight="1">
-      <c r="F31" s="6"/>
+      <c r="F31" s="4"/>
     </row>
     <row r="32" spans="6:6" ht="30" customHeight="1">
-      <c r="F32" s="6"/>
+      <c r="F32" s="4"/>
     </row>
     <row r="33" spans="6:6" ht="30" customHeight="1">
-      <c r="F33" s="6"/>
+      <c r="F33" s="4"/>
     </row>
     <row r="34" spans="6:6" ht="30" customHeight="1">
-      <c r="F34" s="6"/>
+      <c r="F34" s="4"/>
     </row>
     <row r="35" spans="6:6" ht="30" customHeight="1">
-      <c r="F35" s="6"/>
+      <c r="F35" s="4"/>
     </row>
     <row r="36" spans="6:6" ht="30" customHeight="1">
-      <c r="F36" s="6"/>
+      <c r="F36" s="4"/>
     </row>
     <row r="37" spans="6:6" ht="30" customHeight="1">
-      <c r="F37" s="6"/>
+      <c r="F37" s="4"/>
     </row>
     <row r="38" spans="6:6" ht="30" customHeight="1">
-      <c r="F38" s="6"/>
+      <c r="F38" s="4"/>
     </row>
     <row r="39" spans="6:6" ht="30" customHeight="1">
-      <c r="F39" s="6"/>
+      <c r="F39" s="4"/>
     </row>
     <row r="40" spans="6:6" ht="30" customHeight="1">
-      <c r="F40" s="6"/>
+      <c r="F40" s="4"/>
     </row>
     <row r="41" spans="6:6" ht="30" customHeight="1">
-      <c r="F41" s="6"/>
+      <c r="F41" s="4"/>
     </row>
     <row r="42" spans="6:6" ht="30" customHeight="1">
-      <c r="F42" s="6"/>
+      <c r="F42" s="4"/>
     </row>
     <row r="43" spans="6:6" ht="30" customHeight="1">
-      <c r="F43" s="6"/>
+      <c r="F43" s="4"/>
     </row>
     <row r="44" spans="6:6" ht="30" customHeight="1">
-      <c r="F44" s="6"/>
+      <c r="F44" s="4"/>
     </row>
     <row r="45" spans="6:6" ht="30" customHeight="1">
-      <c r="F45" s="6"/>
+      <c r="F45" s="4"/>
     </row>
     <row r="46" spans="6:6" ht="30" customHeight="1">
-      <c r="F46" s="6"/>
+      <c r="F46" s="4"/>
     </row>
     <row r="47" spans="6:6" ht="30" customHeight="1">
-      <c r="F47" s="6"/>
+      <c r="F47" s="4"/>
     </row>
     <row r="48" spans="6:6" ht="30" customHeight="1">
-      <c r="F48" s="6"/>
+      <c r="F48" s="4"/>
     </row>
     <row r="49" spans="6:6" ht="30" customHeight="1">
-      <c r="F49" s="6"/>
+      <c r="F49" s="4"/>
     </row>
     <row r="50" spans="6:6" ht="30" customHeight="1">
-      <c r="F50" s="6"/>
+      <c r="F50" s="4"/>
     </row>
     <row r="51" spans="6:6" ht="30" customHeight="1">
-      <c r="F51" s="6"/>
+      <c r="F51" s="4"/>
     </row>
     <row r="52" spans="6:6" ht="30" customHeight="1">
-      <c r="F52" s="6"/>
+      <c r="F52" s="4"/>
     </row>
     <row r="53" spans="6:6" ht="30" customHeight="1">
-      <c r="F53" s="6"/>
+      <c r="F53" s="4"/>
     </row>
     <row r="54" spans="6:6" ht="30" customHeight="1">
-      <c r="F54" s="6"/>
+      <c r="F54" s="4"/>
     </row>
     <row r="55" spans="6:6" ht="30" customHeight="1">
-      <c r="F55" s="6"/>
+      <c r="F55" s="4"/>
     </row>
     <row r="56" spans="6:6" ht="30" customHeight="1">
-      <c r="F56" s="6"/>
+      <c r="F56" s="4"/>
     </row>
     <row r="57" spans="6:6" ht="30" customHeight="1">
-      <c r="F57" s="6"/>
+      <c r="F57" s="4"/>
     </row>
     <row r="58" spans="6:6" ht="30" customHeight="1">
-      <c r="F58" s="6"/>
+      <c r="F58" s="4"/>
     </row>
     <row r="59" spans="6:6" ht="30" customHeight="1">
-      <c r="F59" s="6"/>
+      <c r="F59" s="4"/>
     </row>
     <row r="60" spans="6:6" ht="30" customHeight="1">
-      <c r="F60" s="6"/>
+      <c r="F60" s="4"/>
     </row>
     <row r="61" spans="6:6" ht="30" customHeight="1">
-      <c r="F61" s="6"/>
+      <c r="F61" s="4"/>
     </row>
     <row r="62" spans="6:6" ht="30" customHeight="1">
-      <c r="F62" s="6"/>
+      <c r="F62" s="4"/>
     </row>
     <row r="63" spans="6:6" ht="30" customHeight="1">
-      <c r="F63" s="6"/>
+      <c r="F63" s="4"/>
     </row>
     <row r="64" spans="6:6" ht="30" customHeight="1">
-      <c r="F64" s="6"/>
+      <c r="F64" s="4"/>
     </row>
     <row r="65" spans="6:6" ht="30" customHeight="1">
-      <c r="F65" s="6"/>
+      <c r="F65" s="4"/>
     </row>
     <row r="66" spans="6:6" ht="30" customHeight="1">
-      <c r="F66" s="6"/>
+      <c r="F66" s="4"/>
     </row>
     <row r="67" spans="6:6" ht="30" customHeight="1">
-      <c r="F67" s="6"/>
+      <c r="F67" s="4"/>
     </row>
     <row r="68" spans="6:6" ht="30" customHeight="1">
-      <c r="F68" s="6"/>
+      <c r="F68" s="4"/>
     </row>
     <row r="69" spans="6:6" ht="30" customHeight="1">
-      <c r="F69" s="6"/>
+      <c r="F69" s="4"/>
     </row>
     <row r="70" spans="6:6" ht="30" customHeight="1">
-      <c r="F70" s="6"/>
+      <c r="F70" s="4"/>
     </row>
     <row r="71" spans="6:6" ht="30" customHeight="1">
-      <c r="F71" s="6"/>
+      <c r="F71" s="4"/>
     </row>
     <row r="72" spans="6:6" ht="30" customHeight="1">
-      <c r="F72" s="6"/>
+      <c r="F72" s="4"/>
     </row>
     <row r="73" spans="6:6" ht="30" customHeight="1">
-      <c r="F73" s="6"/>
+      <c r="F73" s="4"/>
     </row>
     <row r="74" spans="6:6" ht="30" customHeight="1">
-      <c r="F74" s="6"/>
+      <c r="F74" s="4"/>
     </row>
     <row r="75" spans="6:6" ht="30" customHeight="1">
-      <c r="F75" s="6"/>
+      <c r="F75" s="4"/>
     </row>
     <row r="76" spans="6:6" ht="30" customHeight="1">
-      <c r="F76" s="6"/>
+      <c r="F76" s="4"/>
     </row>
     <row r="77" spans="6:6" ht="30" customHeight="1">
-      <c r="F77" s="6"/>
+      <c r="F77" s="4"/>
     </row>
     <row r="78" spans="6:6" ht="30" customHeight="1">
-      <c r="F78" s="6"/>
+      <c r="F78" s="4"/>
     </row>
     <row r="79" spans="6:6" ht="30" customHeight="1">
-      <c r="F79" s="6"/>
+      <c r="F79" s="4"/>
     </row>
     <row r="80" spans="6:6" ht="30" customHeight="1">
-      <c r="F80" s="6"/>
+      <c r="F80" s="4"/>
     </row>
     <row r="81" spans="6:6" ht="30" customHeight="1">
-      <c r="F81" s="6"/>
+      <c r="F81" s="4"/>
     </row>
     <row r="82" spans="6:6" ht="30" customHeight="1">
-      <c r="F82" s="6"/>
+      <c r="F82" s="4"/>
     </row>
     <row r="83" spans="6:6" ht="30" customHeight="1">
-      <c r="F83" s="6"/>
+      <c r="F83" s="4"/>
     </row>
     <row r="84" spans="6:6" ht="30" customHeight="1">
-      <c r="F84" s="6"/>
+      <c r="F84" s="4"/>
     </row>
     <row r="85" spans="6:6" ht="30" customHeight="1">
-      <c r="F85" s="6"/>
+      <c r="F85" s="4"/>
     </row>
     <row r="86" spans="6:6" ht="30" customHeight="1">
-      <c r="F86" s="6"/>
+      <c r="F86" s="4"/>
     </row>
     <row r="87" spans="6:6" ht="30" customHeight="1">
-      <c r="F87" s="6"/>
+      <c r="F87" s="4"/>
     </row>
     <row r="88" spans="6:6" ht="30" customHeight="1">
-      <c r="F88" s="6"/>
+      <c r="F88" s="4"/>
     </row>
     <row r="89" spans="6:6" ht="30" customHeight="1">
-      <c r="F89" s="6"/>
+      <c r="F89" s="4"/>
     </row>
     <row r="90" spans="6:6" ht="30" customHeight="1">
-      <c r="F90" s="6"/>
+      <c r="F90" s="4"/>
     </row>
     <row r="91" spans="6:6" ht="30" customHeight="1">
-      <c r="F91" s="6"/>
+      <c r="F91" s="4"/>
     </row>
     <row r="92" spans="6:6" ht="30" customHeight="1">
-      <c r="F92" s="6"/>
+      <c r="F92" s="4"/>
     </row>
     <row r="93" spans="6:6" ht="30" customHeight="1">
-      <c r="F93" s="6"/>
+      <c r="F93" s="4"/>
     </row>
     <row r="94" spans="6:6" ht="30" customHeight="1">
-      <c r="F94" s="6"/>
+      <c r="F94" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>